<commit_message>
Update GDI6 delivery after local PCB repairs and expose workbook provenance
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R4b3dba798f8d4b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R986dc44458cf47bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R97a6e56178d74db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R3d947918373942cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="Rcb797c81fa974f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rd7407d8848c0406a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Redcc1c959a734276"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48701,4 +48702,120 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF245A81"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="108" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Версия исходных данных</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>28.10.2026 • связь схемы, платы и сметы</x:v>
+      </x:c>
+      <x:c r="B2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="2"/>
+      <x:c r="B4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>Источник</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="str">
+        <x:v>Значение</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="31" t="str">
+        <x:v>Ревизия репозитория</x:v>
+      </x:c>
+      <x:c r="B6" s="32" t="str">
+        <x:v>7c43c2aeba7eb570400faaa0bf9ded6dbfd70f42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>SHA-256 списка соединений</x:v>
+      </x:c>
+      <x:c r="B7" s="32" t="str">
+        <x:v>40a7e18e334463119d4d387b05956dad5c26db4c65daa03aa1706900aad76cf2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="31" t="str">
+        <x:v>SHA-256 платы</x:v>
+      </x:c>
+      <x:c r="B8" s="32" t="str">
+        <x:v>25aa498aa4491da8bf1901736c84a1affb26e64c01c6b818565fbd7b30f6967a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>SHA-256 входов расчёта</x:v>
+      </x:c>
+      <x:c r="B9" s="32" t="str">
+        <x:v>2296e3e03d9bccb5d1f3567d5bca1bfa54ad5288dfa659a95d1e024509864a22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="31" t="str">
+        <x:v>Устанавливаемых позиций</x:v>
+      </x:c>
+      <x:c r="B10" s="32" t="str">
+        <x:v>1047</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>Групп закупки</x:v>
+      </x:c>
+      <x:c r="B11" s="32" t="str">
+        <x:v>149</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>Статус</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>Инженерная версия; производство и работа на двигателе не разрешены.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="31" t="str">
+        <x:v>Пересчёт</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>Синие входы и формулы меняют базовую смету. Нижняя и верхняя оценки сохранены на дату расчёта.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="2"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="2"/>
+      <x:c r="B15" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh GDI6 schematic BOM report and workbook after WBO routing
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R3d947918373942cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="Rcb797c81fa974f48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rd7407d8848c0406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Redcc1c959a734276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R48ff93d8f17f4d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R44839ca6dca742e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R94710b56bd8f43cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Ra84f83d678774cf7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9461,7 +9461,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>1047 устанавливаемых компонентов • 1092 физических позиций • Netlist 40a7e18e33446311…</x:v>
+        <x:v>1047 устанавливаемых компонентов • 1092 физических позиций • Netlist abd9c0533019b981…</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>7c43c2aeba7eb570400faaa0bf9ded6dbfd70f42</x:v>
+        <x:v>403f73faa99a7cadcb141be4e3e5919a52adf5d9</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48756,7 +48756,7 @@
         <x:v>SHA-256 списка соединений</x:v>
       </x:c>
       <x:c r="B7" s="32" t="str">
-        <x:v>40a7e18e334463119d4d387b05956dad5c26db4c65daa03aa1706900aad76cf2</x:v>
+        <x:v>abd9c0533019b9811a75fa73c46c1a9d9b97511d5f858edb2b88ae1e98a87462</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>25aa498aa4491da8bf1901736c84a1affb26e64c01c6b818565fbd7b30f6967a</x:v>
+        <x:v>cf36d99bb312769ed73cdec0149b5d2e6b9fb01143e814fb0145150245b02206</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>2296e3e03d9bccb5d1f3567d5bca1bfa54ad5288dfa659a95d1e024509864a22</x:v>
+        <x:v>1d741375f5095cf418ed8b8723085197dc38ffedfa4f429348f0c630a9bf4fef</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery after VIO bypass and ground routing
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R48ff93d8f17f4d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R44839ca6dca742e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R94710b56bd8f43cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Ra84f83d678774cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rb0fd1c9470fd445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R41a4831c0ed44013"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R49698798da994a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Reccc370405594bca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>403f73faa99a7cadcb141be4e3e5919a52adf5d9</x:v>
+        <x:v>5740487f7f2fd532b013e10d3ce440644a63bc2c</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>cf36d99bb312769ed73cdec0149b5d2e6b9fb01143e814fb0145150245b02206</x:v>
+        <x:v>75e98a2a132238da55b954a4b55d0bde57f14ed8334183e136645a9238173bdf</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>1d741375f5095cf418ed8b8723085197dc38ffedfa4f429348f0c630a9bf4fef</x:v>
+        <x:v>4d6cc62665007d2b9710c2d7f314ab0aee0da2f525754f10ab509ab493561cc7</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery for verified supervisor reset branch
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rb0fd1c9470fd445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R41a4831c0ed44013"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R49698798da994a6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Reccc370405594bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rc8fa462c0c1c47d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R8154c476362c4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R2863deccff944527"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R446ae8119ac34206"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>5740487f7f2fd532b013e10d3ce440644a63bc2c</x:v>
+        <x:v>a048198f9c874eec2f0b0c55c6f3c44e718a0990</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>75e98a2a132238da55b954a4b55d0bde57f14ed8334183e136645a9238173bdf</x:v>
+        <x:v>7e7872186f98b95cc92002db7e7e9ce3789c719f5df7182711846a7bdf729be0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>4d6cc62665007d2b9710c2d7f314ab0aee0da2f525754f10ab509ab493561cc7</x:v>
+        <x:v>78739f0f574e905e50a441b2a03e883519381200649bd1b3c3fcd6f66297e0af</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery after permission gate ground routing
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rc8fa462c0c1c47d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R8154c476362c4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R2863deccff944527"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R446ae8119ac34206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R4ff5be17383044b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="Rf320091fed854329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rfa24eea4d67348e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R0499a6b2e32b4925"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>a048198f9c874eec2f0b0c55c6f3c44e718a0990</x:v>
+        <x:v>6da9fe1d728a6e6d57cdcef2f4606f82a610e0e5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>7e7872186f98b95cc92002db7e7e9ce3789c719f5df7182711846a7bdf729be0</x:v>
+        <x:v>3a6f881bd42b702a6e085e7eddefbcd569296583262431f3ccb02c25484b4f9b</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>78739f0f574e905e50a441b2a03e883519381200649bd1b3c3fcd6f66297e0af</x:v>
+        <x:v>345f5e4cfa79c12252178804b5a47802b933946803ce8a21f493877a5c743cba</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery after MCU and bypass ground connections
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R4ff5be17383044b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="Rf320091fed854329"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rfa24eea4d67348e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R0499a6b2e32b4925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rd85d825e4f334749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R062c2bf8a2aa4b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rf48db068f6234c8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Rc61b0d042ae54d05"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>6da9fe1d728a6e6d57cdcef2f4606f82a610e0e5</x:v>
+        <x:v>78a31c871eee3ce6e5360f6e74e5b3c23f15522c</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>3a6f881bd42b702a6e085e7eddefbcd569296583262431f3ccb02c25484b4f9b</x:v>
+        <x:v>e1887db8720d0945f611a9e5fe935d72f429a886bd382a77690af20472098e17</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>345f5e4cfa79c12252178804b5a47802b933946803ce8a21f493877a5c743cba</x:v>
+        <x:v>944f28eaac93cd5eeaf94268f00524fe16fa83df29807e59240ed5b0c4e83e6c</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery after WBO MCU VDD bypass routing
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="Rd85d825e4f334749"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R062c2bf8a2aa4b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="Rf48db068f6234c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="Rc61b0d042ae54d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R2e1191847e654eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R82ca9da9feb04402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R8a8d358323b944a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R54fe1d91fefb4c99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>78a31c871eee3ce6e5360f6e74e5b3c23f15522c</x:v>
+        <x:v>a73e9d3d07d62842d5e34750fd39db365a8754db</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>e1887db8720d0945f611a9e5fe935d72f429a886bd382a77690af20472098e17</x:v>
+        <x:v>5c1f064233a1a4ba51e6c8f209de365f30a4cd411869d71b7ece4dd3e51703e0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>944f28eaac93cd5eeaf94268f00524fe16fa83df29807e59240ed5b0c4e83e6c</x:v>
+        <x:v>7c1a3991671465b0395f365152d7c6e5d151bc3cd8185eb95b03e3522816988f</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Refresh GDI6 delivery after regulator feed and ground returns
</commit_message>
<xml_diff>
--- a/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
+++ b/Power8GDI/docs/reports/2026-10-28-gdi6/Sport_GDI6_BOM_and_cost.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R2e1191847e654eea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R82ca9da9feb04402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R8a8d358323b944a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R54fe1d91fefb4c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" r:id="R9b805326a0bc4877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Закупка" sheetId="2" r:id="R050fc0cb9d0a4a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM по позициям" sheetId="3" r:id="R239471cca7114346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версия исходных данных" sheetId="4" r:id="R5b0ef6a6264543b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48748,7 +48748,7 @@
         <x:v>Ревизия репозитория</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>a73e9d3d07d62842d5e34750fd39db365a8754db</x:v>
+        <x:v>965ebbca7fff19c6c666d253daeea0b1a29b4485</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -48764,7 +48764,7 @@
         <x:v>SHA-256 платы</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>5c1f064233a1a4ba51e6c8f209de365f30a4cd411869d71b7ece4dd3e51703e0</x:v>
+        <x:v>638900cd40914d65b20f752ccf2698f53bb84e6ac96d56a0a211c24fb287576f</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -48772,7 +48772,7 @@
         <x:v>SHA-256 входов расчёта</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
-        <x:v>7c1a3991671465b0395f365152d7c6e5d151bc3cd8185eb95b03e3522816988f</x:v>
+        <x:v>bb98582a0f4a27693974598e195498f8d37f1e503c11f775f4ca3f96d082863d</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">

</xml_diff>